<commit_message>
feat(survey): update excel responses with 25 survey rows
</commit_message>
<xml_diff>
--- a/myntra-growth-app/Online Fashion Shopping & Browsing Habits Survey (2026) (Responses).xlsx
+++ b/myntra-growth-app/Online Fashion Shopping & Browsing Habits Survey (2026) (Responses).xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ujjaw\Desktop\Graduation Project 2\myntra-growth-app\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FEFF897-2978-4466-890E-FA245D80FFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -241,11 +247,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -283,13 +289,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -327,7 +341,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -361,6 +375,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -395,9 +410,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -570,11 +586,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="255.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="101.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="80.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="129.1328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="134.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="112.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="96.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="107" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="60.3984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -615,9 +646,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>46254.98774202546</v>
+        <v>46254.987742025463</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -650,9 +681,9 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
-        <v>46255.39758182871</v>
+        <v>46255.397581828707</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -685,9 +716,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
-        <v>46255.53099229166</v>
+        <v>46255.530992291657</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -723,9 +754,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
-        <v>46255.53286541667</v>
+        <v>46255.532865416673</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -761,9 +792,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
-        <v>46255.72072311342</v>
+        <v>46255.720723113423</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -799,9 +830,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
-        <v>46255.7209153588</v>
+        <v>46255.720915358797</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -834,9 +865,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
-        <v>46255.76400854166</v>
+        <v>46255.764008541657</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
@@ -869,9 +900,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
-        <v>46255.78759629629</v>
+        <v>46255.787596296293</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -904,7 +935,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>46255.93399409722</v>
       </c>
@@ -945,7 +976,7 @@
         <v>9496336815</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>46256.42664351852</v>
       </c>
@@ -986,9 +1017,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
-        <v>46256.61469907407</v>
+        <v>46256.614699074067</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
@@ -1027,9 +1058,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
-        <v>46257.47260416667</v>
+        <v>46257.472604166673</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1065,9 +1096,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
-        <v>46257.67061342593</v>
+        <v>46257.670613425929</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
@@ -1103,9 +1134,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
-        <v>46258.39600694444</v>
+        <v>46258.396006944437</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
@@ -1144,9 +1175,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
-        <v>46258.5505787037</v>
+        <v>46258.550578703696</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
@@ -1185,7 +1216,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>46258.77783564815</v>
       </c>
@@ -1223,9 +1254,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
-        <v>46259.4621412037</v>
+        <v>46259.462141203701</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
@@ -1264,9 +1295,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
-        <v>46259.64043981482</v>
+        <v>46259.640439814822</v>
       </c>
       <c r="B19" t="s">
         <v>13</v>
@@ -1302,9 +1333,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
-        <v>46260.45194444444</v>
+        <v>46260.451944444438</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -1343,9 +1374,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
-        <v>46260.71909722222</v>
+        <v>46260.719097222223</v>
       </c>
       <c r="B21" t="s">
         <v>13</v>
@@ -1381,9 +1412,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
-        <v>46261.50298611111</v>
+        <v>46261.502986111111</v>
       </c>
       <c r="B22" t="s">
         <v>13</v>
@@ -1422,9 +1453,9 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
-        <v>46261.81645833333</v>
+        <v>46261.816458333327</v>
       </c>
       <c r="B23" t="s">
         <v>13</v>
@@ -1460,7 +1491,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <v>46262.47146990741</v>
       </c>
@@ -1501,9 +1532,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
-        <v>46262.61819444445</v>
+        <v>46262.618194444447</v>
       </c>
       <c r="B25" t="s">
         <v>13</v>
@@ -1542,9 +1573,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
-        <v>46262.88237268518</v>
+        <v>46262.882372685177</v>
       </c>
       <c r="B26" t="s">
         <v>13</v>

</xml_diff>